<commit_message>
Actualizar vigilancia normativa 2026-08-28 21:51 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E543"/>
+  <dimension ref="A1:E704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15077,6 +15077,4353 @@
         </is>
       </c>
     </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>ir al contenido</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/decretos-2026/decretos-enero-2026/#contentBox</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0124 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0124 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0123 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0123 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0121 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0121 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0120 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0120 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0118 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0118 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0115 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0115 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0114 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0114 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0113 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0113 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0110 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0110 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0108 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0108 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0107 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0107 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0106 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0106 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0105 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0105 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0104 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0104 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0103 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0103 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0102 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0102 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0101 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0101 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0100 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0100 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0099 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0099 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0098 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0098 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0097 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0097 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0096 DEL 30 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0096 DEL 30 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0093 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0093 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0092 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0092 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0089 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0089 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0088 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0088 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0087 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0087 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0085 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0085 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0084 DEL 29 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0084 DEL 29 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0080 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0080 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0079 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0079 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0078 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0078 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0076 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0076 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0073 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0073 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0072 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0072 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0071 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0071 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0069 DEL 27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0069 DEL 27 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0065 DEL 26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0065 DEL 26 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0064 DEL 26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0064 DEL 26 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0063 DEL 26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0063 DEL 26 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0061 DEL 26 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0061 DEL 26 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>23 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0059 DEL 23 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0059 DEL 23 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>23 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0057 DEL 23 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0057 DEL 23 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0054 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0054 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0053 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0053 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0052 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0052 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0051 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0051 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0050 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0050 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0049 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0049 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0048 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0048 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0047 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0047 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0046 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0046 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0045 DEL 22 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0045 DEL 22 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0044 DEL 21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0044 DEL 21 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0042 DEL 21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0042 DEL 21 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0041 DEL 21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0041 DEL 21 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0040 DEL 21 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0040 DEL 21 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0039 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0039 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0038 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0038 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0037 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0037 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0036 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0036 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0035 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0035 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0034 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0034 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0033 DEL 20 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0033 DEL 20 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>19 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0030 DEL 19 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0030 DEL 19 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>19 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0029 DEL 19 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0029 DEL 19 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0023 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0023 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0022 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0022 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0021 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0021 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0020 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0020 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0019 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0019 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0018 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0018 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0017 DEL 15 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0017 DEL 15 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>14 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0011 DEL 14 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0011 DEL 14 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>14 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0013 DEL 14 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0013 DEL 14 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>13 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0009 DEL 13 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0009 DEL 13 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Enero 2026</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>9 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>DECRETO No. 0004 DEL 9 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 0004 DEL 9 DE ENERO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>27 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1329 DEL 27 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1329 DEL 27 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1327 DEL 26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1327 DEL 26 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1325 DEL 26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1325 DEL 26 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1323 DEL 26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1323 DEL 26 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1322 DEL 26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1322 DEL 26 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1321 DEL 26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1321 DEL 26 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1320 DEL 26 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1320 DEL 26 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1317 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1317 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1316 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1316 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1312 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1312 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1311 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1311 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1309 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1309 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1308 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1308 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1306 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1306 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1305 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1305 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1304 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1304 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1303 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1303 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1302 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1302 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1299 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1299 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1298 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1298 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1297 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1297 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1296 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1296 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1295 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1295 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1294 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1294 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1292 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1292 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1291 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1291 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1290 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1290 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1288 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1288 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1287 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1287 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1284 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1284 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1283 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1283 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1282 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1282 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1281 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1281 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1280 DEL 25 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1280 DEL 25 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>4 DE MAYO DE 2026</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>ir al contenido</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/circulares/#contentBox</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>4 DE MAYO DE 2026</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>CIR26-00000027 - GFPU 4 de Mayo 2026</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIR26-00000027 _ GFPU.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>27 DE ENERO DE 2026</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>CIR26-00000007-GFPU 27 de enero 2026</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIR26-00000007 _ GFPU.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>04 DE SEPTIEMBRE DE 2024</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Circular 24-00000037 del 04 de septiembre de 2024, D</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIR25-00000037 _ GFPU 04-09-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2025</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>CIRCULAR 04 DEL 25 DE AGOSTO DE 2025</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 04 DEL 25 DE AGOSTO DE 2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>25 DE AGOSTO DE 2025</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>CIRCULAR 03 DEL 25 DE AGOSTO DE 2025</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 03 DEL 25 DE AGOSTO DE 2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>28 DE NOVIEMBRE DE 2024</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>CIR24-00000085 del 28 de noviembre de 2024</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIR24-00000085 _ GFPU_tramite_fin_de_a_o_ENTIDADES.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>22 DE MAYO DE 2024</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>CIR24-00000032 del 22 de mayo de 2024.</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIR24-00000032 _ Directrices-tramite-autorizacioncomisiones-rama-ejecutiva.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>22 DE NOVIEMBRE DE 2023</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>CIRCULAR No 05 DEL 22 DE NOVIEMBRE DE 2023</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR No 05 DEL 22 DE NOVIEMBRE DE 2023.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>30 DE AGOSTO DE 2023</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>CIRCULAR No 04 DEL 30 DE AGOSTO DE 2023</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR No 04 DEL 30 DE AGOSTO DE 2023.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>30 DE MAYO DE 2023</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>CIRCULAR No 03 DEL 30 DE MAYO DE 2023</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR No 03 DEL 30 DE MAYO DE 2023.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>29 DE MARZO DE 2023</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>CIRCULAR No 02 DEL 29 DE MARZO DE 2023</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR No 02 DEL 29 DE MARZO DE 2023.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>29 DE MARZO DE 2023</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>CIRCULAR No 01 DEL 29 DE MARZO DE 2023</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR No 01 DEL 29 DE MARZO DE 2023.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>10 DE OCTUBRE DE 2022</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>CIRCULAR 06 DEL 10 DE OCTUBRE DE 2022</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 06 DEL 10 DE OCTUBRE DE 2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>14 DE SEPTIEMBRE DE 2022</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>CIRCULAR 05 DEL 14 DE SEPTIEMBRE DE 2022</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 05 DEL 14 DE SEPTIEMBRE DE 2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>6 DE JULIO DE 2022</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>CIRCULAR 04 DEL 6 DE JULIO DE 2022</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 04 DEL 6 DE JULIO DE 2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>6 DE JUNIO DE 2022</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>CIRCULAR 03 DEL 6 DE JUNIO DE 2022</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 03 DEL 6 DE JUNIO DE 2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>1 DE JUNIO DE 2022</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>CIRCULAR 02 DEL 1 DE JUNIO DE 2022</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 02 DEL 1 DE JUNIO DE 2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>17 DE FEBRERO DE 2022</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>CIRCULAR 01 DEL 17 DE FEBRERO DE 2022</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 01 DEL 17 DE FEBRERO DE 2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>11 DE NOVIEMBRE DE 2021</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>CIRCULAR 05 DEL 11 DE NOVIEMBRE DE 2021</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 05 DEL 11 DE NOVIEMBRE DE 2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>4 DE NOVIEMBRE DE 2021</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>CIRCULAR 04 DEL 4 DE NOVIEMBRE DE 2021</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 04 DEL 4 DE NOVIEMBRE DE 2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>11 DE JUNIO DE 2021</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>CIRCULAR PRESIDENCIA 01 DEL 11 DE JUNIO DE 2021</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR PRESIDENCIA 01 DEL 11 DE JUNIO DE 2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>13 DE ABRIL DE 2021</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>CIRCULAR 03 DEL 13 DE ABRIL DE 2021</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 03 DEL 13 DE ABRIL DE 2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>13 DE ABRIL DE 2021</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>CIRCULAR 02 DEL 13 DE ABRIL DE 2021</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 02 DEL 13 DE ABRIL DE 2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>24 DE FEBRERO DE 2021</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Circular 01 del 24 de febrero de 2021</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/Circular 01 del 24 de febrero de 2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>09 DE OCTUBRE DE 2020</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>CIRCULAR 01 DEL 09 DE OCTUBRE DE 2020</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 01 DEL 09 DE OCTUBRE DE 2020.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>11 DE MARZO DE 2020</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Circular CIR20-00000018 de 11 de marzo de 2020</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/Circular20-00000018-comisionesext-covid19.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>18 DE DICIEMBRE DE 2019</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>CIRCULAR PRESIDENCIAL N° 03 DEL 18 DE DICIEMBRE DE 2019</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR PRESIDENCIAL N° 03 DEL 18 DE DICIEMBRE DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>29 DE NOVIEMBRE DE 2019</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 06 DEL 29 DE NOVIEMBRE DE 2019</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 06 DEL 29 DE NOVIEMBRE DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>18 DE OCTUBRE DE 2019</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 02 DEL 18 DE OCTUBRE DE 2019</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 02 DEL 18 DE OCTUBRE DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>30 DE AGOSTO DE 2019</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 05 DEL 30 DE AGOSTO DE 2019</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 05 DEL 30 DE AGOSTO DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>08 DE JULIO DE 2019</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 04 DEL 08 DE JULIO DE 2019</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 04 DEL 08 DE JULIO DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>17 DE JUNIO DE 2019</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 03 DEL 17 DE JUNIO DE 2019</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 03 DEL 17 DE JUNIO DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>13 DE JUNIO DE 2019</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 02 DEL 13 DE JUNIO DE 2019</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 02 DEL 13 DE JUNIO DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>22 DE MARZO DE 2019</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>CIRCULAR N° 01 DEL 22 DE MARZO DE 2019</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR N° 01 DEL 22 DE MARZO DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>15 DE ENERO DE 2019</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>CIRCULAR PRESIDENCIAL N° 01 DEL 15 DE ENERO DE 2019</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR PRESIDENCIAL N° 01 DEL 15 DE ENERO DE 2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>20 DE NOVIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>CIRCULAR PRESIDENCIAL 01 DEL 20 DE NOVIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR PRESIDENCIAL 01 DEL 20 DE NOVIEMBRE DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>21 DE NOVIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 07 DEL 21 DE NOVIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 07 DEL 21 DE NOVIEMBRE DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>17 DE OCTUBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 06 DEL 17 DE OCTUBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 06 DEL 17 DE OCTUBRE DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>21 DE SEPTIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 05 DEL 21 DE SEPTIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 05 DEL 21 DE SEPTIEMBRE DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>21 DE SEPTIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 04 DEL 21 DE SEPTIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 04 DEL 21 DE SEPTIEMBRE DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>13 DE SEPTIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 03 DEL 13 DE SEPTIEMBRE DE 2018</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 03 DEL 13 DE SEPTIEMBRE DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>27 DE AGOSTO DE 2018</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Circular No. 0012 del 27 de agosto de 2018</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/circular-0012-27-agosto-2018-factura-electronica.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>17 DE AGOSTO DE 2018</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 02 DEL 17 DE AGOSTO DE 2018</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 02 DEL 17 DE AGOSTO DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>01 DE FEBRERO DE 2018</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 01 DEL 01 DE FEBRERO DE 2018</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 01 DEL 01 DE FEBRERO DE 2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>27 DE OCTUBRE DE 2017</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>CIRCULAR 03 DEL 27 DE OCTUBRE DE 2017</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 03 DEL 27 DE OCTUBRE DE 2017.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>26 DE OCTUBRE DE 2017</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA 01 DEL 26 DE OCTUBRE DE 2017</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA 01 DEL 26 DE OCTUBRE DE 2017.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>20 DE OCTUBRE DE 2017</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>CIRCULAR 02 DEL 20 DE OCTUBRE DE 2017</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 02 DEL 20 DE OCTUBRE DE 2017.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-08-28 21:51</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>10 DE JULIO DE 2017</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>CIRCULAR 01 DEL 10 DE JULIO DE 2017</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR 01 DEL 10 DE JULIO DE 2017.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-01 13:04 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1577"/>
+  <dimension ref="A1:E1585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42995,6 +42995,222 @@
         </is>
       </c>
     </row>
+    <row r="1578">
+      <c r="A1578" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1578" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1578" t="inlineStr">
+        <is>
+          <t>31 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1578" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1347 DEL 31 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1578" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1347 DEL 31 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1579" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1579" t="inlineStr">
+        <is>
+          <t>31 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1579" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1346 DEL 31 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1579" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1346 DEL 31 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1580" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1580" t="inlineStr">
+        <is>
+          <t>28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1580" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1339 DEL 28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1580" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1339 DEL 28 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1581" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1581" t="inlineStr">
+        <is>
+          <t>28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1581" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1338 DEL 28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1581" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1338 DEL 28 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1582" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1582" t="inlineStr">
+        <is>
+          <t>28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1582" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1337 DEL 28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1582" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1337 DEL 28 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1583" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1583" t="inlineStr">
+        <is>
+          <t>28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1583" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1334 DEL 28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1583" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1334 DEL 28 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1584" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1584" t="inlineStr">
+        <is>
+          <t>28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1584" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1332 DEL 28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1584" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1332 DEL 28 DE AGOSTO DE 2026 1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:04</t>
+        </is>
+      </c>
+      <c r="B1585" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1585" t="inlineStr">
+        <is>
+          <t>28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1585" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1331 DEL 28 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1585" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1331 DEL 28 DE AGOSTO DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-04 13:03 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1585"/>
+  <dimension ref="A1:E1586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43211,6 +43211,33 @@
         </is>
       </c>
     </row>
+    <row r="1586">
+      <c r="A1586" t="inlineStr">
+        <is>
+          <t>2026-09-04 13:03</t>
+        </is>
+      </c>
+      <c r="B1586" t="inlineStr">
+        <is>
+          <t>Presidencia - Decretos Agosto 2026</t>
+        </is>
+      </c>
+      <c r="C1586" t="inlineStr">
+        <is>
+          <t>31 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1586" t="inlineStr">
+        <is>
+          <t>DECRETO No. 1348 DEL 31 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="E1586" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/DECRETO No. 1348 DEL 31 DE AGOSTO DE 2026 1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-06 13:03 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1586"/>
+  <dimension ref="A1:E1594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43238,6 +43238,222 @@
         </is>
       </c>
     </row>
+    <row r="1587">
+      <c r="A1587" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1587" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1587" t="inlineStr">
+        <is>
+          <t>3 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1587" t="inlineStr">
+        <is>
+          <t>LEY No. 2632 DEL 3 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1587" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2632 DEL 3 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1588" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1588" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1588" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 371 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1588" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 371 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1589" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1589" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1589" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 370 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1589" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 370 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1590" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1590" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1590" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 369 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1590" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 369 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1591" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1591" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1591" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 368 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1591" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 368 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1592" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 367 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1592" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 367 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1593" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 366 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1593" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 366 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:03</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr">
+        <is>
+          <t>03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1594" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 365 DEL 03 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1594" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 365 DEL 03 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>